<commit_message>
updated logs, updated file conversion/processing guide
</commit_message>
<xml_diff>
--- a/Research Logs/Matt/Matt Baker - Week 8 Research Log.xlsx
+++ b/Research Logs/Matt/Matt Baker - Week 8 Research Log.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RecoveryAdmin\Documents\BHB-Capstone\Research Logs\Matt\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A542A26F-E342-4ACB-BB98-51BF39BD088D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B43890F-AAA5-423C-A27A-22910FF11407}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5475" yWindow="5340" windowWidth="23295" windowHeight="13320" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4755" yWindow="1950" windowWidth="30180" windowHeight="13320" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Research template" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="119">
   <si>
     <t>Date</t>
   </si>
@@ -423,6 +423,39 @@
   </si>
   <si>
     <t>There was not too much to learn beyond what I learned attempting to practically employ them in the Kali environment</t>
+  </si>
+  <si>
+    <t>How to do bash scripting, to make a script that automatically applies commands to different foremost file types.</t>
+  </si>
+  <si>
+    <t>Google, YouTube
+https://stackoverflow.com/questions/37052899/what-is-the-preferred-method-to-echo-a-blank-line-in-a-shell-script
+https://www.youtube.com/watch?v=usyzSMFfUTg
+https://www.youtube.com/watch?v=KG97VzMjfMg</t>
+  </si>
+  <si>
+    <t>Watching/Searching/
+Reading</t>
+  </si>
+  <si>
+    <t>Learned/Relearned how to creat and call variables/arguments, call the correct interpreter, execute bash scripts, I then seek to find out if python scripting is better/possible to do what I want this program to do as it was suggested by bryce.</t>
+  </si>
+  <si>
+    <t>How to do python scripting in Linux to the degree that I can automate the scanning of carved files.</t>
+  </si>
+  <si>
+    <t>Watching/Reading</t>
+  </si>
+  <si>
+    <t>Viewed select videos from this playlist:
+https://www.youtube.com/watch?v=G7koz-Ma6I8&amp;list=PLT98CRl2KxKGIazPd2nQEPbG7sQpT8LEj&amp;index=9
+Read from select sources on specific issues
+https://www.w3schools.com/python/ref_os_chdir.asp
+https://www.w3schools.com/python/python_string_formatting.asp
+https://stackoverflow.com/questions/72024970/how-would-i-store-the-shell-command-output-to-a-variable-in-python</t>
+  </si>
+  <si>
+    <t>Learned/relearned parts of python relevant to the script I want to make. How to do functions, how to use os commands from python script, how to change directories. I learned how to use f-strings to pass in variables through "placeholders". I also learned how to read commands and retrieve their output as variables with subprocess.</t>
   </si>
 </sst>
 </file>
@@ -808,7 +841,7 @@
       </c>
       <c r="D2" s="5">
         <f>ROUNDDOWN(SUM(C6:C499)/60,0)</f>
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="E2" t="s">
         <v>8</v>
@@ -820,7 +853,7 @@
       </c>
       <c r="D3" s="5">
         <f>ROUND(MOD(SUM(C6:C499),60),0)</f>
-        <v>45</v>
+        <v>15</v>
       </c>
     </row>
     <row r="5" spans="2:7" x14ac:dyDescent="0.25">
@@ -1491,11 +1524,45 @@
         <v>109</v>
       </c>
     </row>
-    <row r="47" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="E47" s="1"/>
-    </row>
-    <row r="48" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="E48" s="1"/>
+    <row r="47" spans="2:7" ht="75" x14ac:dyDescent="0.25">
+      <c r="B47" s="3">
+        <v>46271</v>
+      </c>
+      <c r="C47">
+        <v>30</v>
+      </c>
+      <c r="D47" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="E47" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="F47" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="G47" s="1" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="48" spans="2:7" ht="90" x14ac:dyDescent="0.25">
+      <c r="B48" s="3">
+        <v>46271</v>
+      </c>
+      <c r="C48">
+        <v>120</v>
+      </c>
+      <c r="D48" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="E48" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="F48" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="G48" s="1" t="s">
+        <v>117</v>
+      </c>
     </row>
   </sheetData>
   <hyperlinks>

</xml_diff>